<commit_message>
Update template - Remove cell addresses
</commit_message>
<xml_diff>
--- a/config/Gait Lab Physical Exam Template 2026.xlsx
+++ b/config/Gait Lab Physical Exam Template 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://autuni-my.sharepoint.com/personal/em19830_aut_ac_nz/Documents/HRRI Gait lab/Motion Connect Databank/PyCharm/databank_export/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="53" documentId="11_8ED2F9A0AE62749DF43FEA088F4C3829D5A37722" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3FEBF671-2FE4-485F-8C21-1F2551BB24E0}"/>
+  <xr:revisionPtr revIDLastSave="57" documentId="11_8ED2F9A0AE62749DF43FEA088F4C3829D5A37722" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44ECFE8D-95DC-46C3-BCCF-23EB57E6681F}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="660" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
@@ -1447,66 +1447,34 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1517,9 +1485,18 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1529,11 +1506,6 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1546,41 +1518,69 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="277">
@@ -1878,6 +1878,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2188,72 +2192,72 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="81" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
+      <c r="B1" s="82"/>
+      <c r="C1" s="82"/>
+      <c r="D1" s="82"/>
+      <c r="E1" s="82"/>
+      <c r="F1" s="82"/>
+      <c r="G1" s="82"/>
+      <c r="H1" s="82"/>
+      <c r="I1" s="82"/>
+      <c r="J1" s="82"/>
     </row>
     <row r="2" spans="1:10" ht="18" x14ac:dyDescent="0.35">
-      <c r="A2" s="36"/>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
+      <c r="A2" s="83"/>
+      <c r="B2" s="83"/>
+      <c r="C2" s="83"/>
+      <c r="D2" s="83"/>
+      <c r="E2" s="83"/>
+      <c r="F2" s="83"/>
+      <c r="G2" s="83"/>
+      <c r="H2" s="83"/>
+      <c r="I2" s="83"/>
+      <c r="J2" s="83"/>
     </row>
     <row r="3" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="37"/>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
-      <c r="F3" s="37"/>
-      <c r="G3" s="38" t="s">
+      <c r="B3" s="84"/>
+      <c r="C3" s="84"/>
+      <c r="D3" s="84"/>
+      <c r="E3" s="84"/>
+      <c r="F3" s="84"/>
+      <c r="G3" s="85" t="s">
         <v>104</v>
       </c>
-      <c r="H3" s="38"/>
-      <c r="I3" s="37"/>
-      <c r="J3" s="39"/>
+      <c r="H3" s="85"/>
+      <c r="I3" s="84"/>
+      <c r="J3" s="86"/>
     </row>
     <row r="4" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B4" s="30"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="32" t="s">
+      <c r="B4" s="79"/>
+      <c r="C4" s="76"/>
+      <c r="D4" s="80" t="s">
         <v>89</v>
       </c>
-      <c r="E4" s="32"/>
+      <c r="E4" s="80"/>
       <c r="F4" s="5"/>
-      <c r="G4" s="32" t="s">
+      <c r="G4" s="80" t="s">
         <v>2</v>
       </c>
-      <c r="H4" s="32"/>
-      <c r="I4" s="30"/>
-      <c r="J4" s="33"/>
+      <c r="H4" s="80"/>
+      <c r="I4" s="79"/>
+      <c r="J4" s="77"/>
     </row>
     <row r="5" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="40"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
+      <c r="B5" s="75"/>
+      <c r="C5" s="76"/>
+      <c r="D5" s="76"/>
       <c r="E5" s="6" t="s">
         <v>4</v>
       </c>
@@ -2262,18 +2266,18 @@
         <v>5</v>
       </c>
       <c r="H5" s="8"/>
-      <c r="I5" s="31"/>
-      <c r="J5" s="33"/>
+      <c r="I5" s="76"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="41"/>
-      <c r="C6" s="41"/>
-      <c r="D6" s="41"/>
-      <c r="E6" s="41"/>
-      <c r="F6" s="41"/>
+      <c r="B6" s="78"/>
+      <c r="C6" s="78"/>
+      <c r="D6" s="78"/>
+      <c r="E6" s="78"/>
+      <c r="F6" s="78"/>
       <c r="G6" s="10" t="s">
         <v>7</v>
       </c>
@@ -2287,124 +2291,82 @@
       <c r="A7" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="42" t="s">
+      <c r="B7" s="71" t="s">
         <v>90</v>
       </c>
-      <c r="C7" s="43"/>
-      <c r="D7" s="42" t="s">
+      <c r="C7" s="72"/>
+      <c r="D7" s="71" t="s">
         <v>91</v>
       </c>
-      <c r="E7" s="43"/>
+      <c r="E7" s="72"/>
       <c r="F7" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G7" s="42" t="s">
+      <c r="G7" s="71" t="s">
         <v>90</v>
       </c>
-      <c r="H7" s="43"/>
-      <c r="I7" s="44" t="s">
+      <c r="H7" s="72"/>
+      <c r="I7" s="73" t="s">
         <v>91</v>
       </c>
-      <c r="J7" s="45"/>
+      <c r="J7" s="74"/>
     </row>
     <row r="8" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="64" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>B8</v>
-      </c>
-      <c r="C8" s="65"/>
-      <c r="D8" s="64" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>D8</v>
-      </c>
-      <c r="E8" s="65"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="34"/>
       <c r="F8" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="64" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>G8</v>
-      </c>
-      <c r="H8" s="65"/>
-      <c r="I8" s="64" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>I8</v>
-      </c>
-      <c r="J8" s="65"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="34"/>
+      <c r="I8" s="33"/>
+      <c r="J8" s="34"/>
     </row>
     <row r="9" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="B9" s="64" t="str">
-        <f t="shared" ref="B9:B13" si="0">ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>B9</v>
-      </c>
-      <c r="C9" s="65"/>
-      <c r="D9" s="64" t="str">
-        <f t="shared" ref="D9:D11" si="1">ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>D9</v>
-      </c>
-      <c r="E9" s="65"/>
+      <c r="B9" s="33"/>
+      <c r="C9" s="34"/>
+      <c r="D9" s="33"/>
+      <c r="E9" s="34"/>
       <c r="F9" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="64" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>G9</v>
-      </c>
-      <c r="H9" s="65"/>
-      <c r="I9" s="64" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>I9</v>
-      </c>
-      <c r="J9" s="65"/>
+      <c r="G9" s="33"/>
+      <c r="H9" s="34"/>
+      <c r="I9" s="33"/>
+      <c r="J9" s="34"/>
     </row>
     <row r="10" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="B10" s="64" t="str">
-        <f t="shared" si="0"/>
-        <v>B10</v>
-      </c>
-      <c r="C10" s="65"/>
-      <c r="D10" s="64" t="str">
-        <f t="shared" si="1"/>
-        <v>D10</v>
-      </c>
-      <c r="E10" s="65"/>
+      <c r="B10" s="33"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="33"/>
+      <c r="E10" s="34"/>
       <c r="F10" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="G10" s="64" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>G10</v>
-      </c>
-      <c r="H10" s="65"/>
-      <c r="I10" s="64" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>I10</v>
-      </c>
-      <c r="J10" s="65"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="34"/>
+      <c r="I10" s="33"/>
+      <c r="J10" s="34"/>
     </row>
     <row r="11" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="17" t="s">
         <v>87</v>
       </c>
-      <c r="B11" s="64" t="str">
-        <f t="shared" si="0"/>
-        <v>B11</v>
-      </c>
-      <c r="C11" s="65"/>
-      <c r="D11" s="64" t="str">
-        <f t="shared" si="1"/>
-        <v>D11</v>
-      </c>
-      <c r="E11" s="65"/>
+      <c r="B11" s="33"/>
+      <c r="C11" s="34"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="34"/>
       <c r="F11" s="15" t="s">
         <v>19</v>
       </c>
@@ -2440,163 +2402,67 @@
       <c r="F12" s="17" t="s">
         <v>99</v>
       </c>
-      <c r="G12" s="18" t="str">
-        <f t="shared" ref="C12:J20" si="2">ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>G12</v>
-      </c>
-      <c r="H12" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>H12</v>
-      </c>
-      <c r="I12" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>I12</v>
-      </c>
-      <c r="J12" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>J12</v>
-      </c>
+      <c r="G12" s="18"/>
+      <c r="H12" s="18"/>
+      <c r="I12" s="18"/>
+      <c r="J12" s="18"/>
     </row>
     <row r="13" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="18" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>B13</v>
-      </c>
-      <c r="C13" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>C13</v>
-      </c>
-      <c r="D13" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>D13</v>
-      </c>
-      <c r="E13" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>E13</v>
-      </c>
+      <c r="B13" s="18"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18"/>
       <c r="F13" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="G13" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>G13</v>
-      </c>
-      <c r="H13" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>H13</v>
-      </c>
-      <c r="I13" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>I13</v>
-      </c>
-      <c r="J13" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>J13</v>
-      </c>
+      <c r="G13" s="18"/>
+      <c r="H13" s="18"/>
+      <c r="I13" s="18"/>
+      <c r="J13" s="18"/>
     </row>
     <row r="14" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="18" t="str">
-        <f t="shared" ref="B14:B18" si="3">ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>B14</v>
-      </c>
-      <c r="C14" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>C14</v>
-      </c>
-      <c r="D14" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>D14</v>
-      </c>
-      <c r="E14" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>E14</v>
-      </c>
+      <c r="B14" s="18"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
       <c r="F14" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="G14" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>G14</v>
-      </c>
-      <c r="H14" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>H14</v>
-      </c>
-      <c r="I14" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>I14</v>
-      </c>
-      <c r="J14" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>J14</v>
-      </c>
+      <c r="G14" s="18"/>
+      <c r="H14" s="18"/>
+      <c r="I14" s="18"/>
+      <c r="J14" s="18"/>
     </row>
     <row r="15" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="B15" s="18" t="str">
-        <f t="shared" si="3"/>
-        <v>B15</v>
-      </c>
-      <c r="C15" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>C15</v>
-      </c>
-      <c r="D15" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>D15</v>
-      </c>
-      <c r="E15" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>E15</v>
-      </c>
+      <c r="B15" s="18"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
       <c r="F15" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="G15" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>G15</v>
-      </c>
-      <c r="H15" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>H15</v>
-      </c>
-      <c r="I15" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>I15</v>
-      </c>
-      <c r="J15" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>J15</v>
-      </c>
+      <c r="G15" s="18"/>
+      <c r="H15" s="18"/>
+      <c r="I15" s="18"/>
+      <c r="J15" s="18"/>
     </row>
     <row r="16" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="18" t="str">
-        <f t="shared" si="3"/>
-        <v>B16</v>
-      </c>
-      <c r="C16" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>C16</v>
-      </c>
-      <c r="D16" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>D16</v>
-      </c>
-      <c r="E16" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>E16</v>
-      </c>
+      <c r="B16" s="18"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="18"/>
       <c r="F16" s="15" t="s">
         <v>26</v>
       </c>
@@ -2617,81 +2483,33 @@
       <c r="A17" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="18" t="str">
-        <f t="shared" si="3"/>
-        <v>B17</v>
-      </c>
-      <c r="C17" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>C17</v>
-      </c>
-      <c r="D17" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>D17</v>
-      </c>
-      <c r="E17" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>E17</v>
-      </c>
+      <c r="B17" s="18"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18"/>
       <c r="F17" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="G17" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>G17</v>
-      </c>
-      <c r="H17" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>H17</v>
-      </c>
-      <c r="I17" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>I17</v>
-      </c>
-      <c r="J17" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>J17</v>
-      </c>
+      <c r="G17" s="18"/>
+      <c r="H17" s="18"/>
+      <c r="I17" s="18"/>
+      <c r="J17" s="18"/>
     </row>
     <row r="18" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="18" t="str">
-        <f t="shared" si="3"/>
-        <v>B18</v>
-      </c>
-      <c r="C18" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>C18</v>
-      </c>
-      <c r="D18" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>D18</v>
-      </c>
-      <c r="E18" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>E18</v>
-      </c>
+      <c r="B18" s="18"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
       <c r="F18" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="G18" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>G18</v>
-      </c>
-      <c r="H18" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>H18</v>
-      </c>
-      <c r="I18" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>I18</v>
-      </c>
-      <c r="J18" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>J18</v>
-      </c>
+      <c r="G18" s="18"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="18"/>
+      <c r="J18" s="18"/>
     </row>
     <row r="19" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="14" t="s">
@@ -2712,83 +2530,35 @@
       <c r="F19" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="G19" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>G19</v>
-      </c>
-      <c r="H19" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>H19</v>
-      </c>
-      <c r="I19" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>I19</v>
-      </c>
-      <c r="J19" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>J19</v>
-      </c>
+      <c r="G19" s="18"/>
+      <c r="H19" s="18"/>
+      <c r="I19" s="18"/>
+      <c r="J19" s="18"/>
     </row>
     <row r="20" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="17" t="s">
         <v>93</v>
       </c>
-      <c r="B20" s="18" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>B20</v>
-      </c>
-      <c r="C20" s="18" t="str">
-        <f t="shared" ref="C20:E24" si="4">ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>C20</v>
-      </c>
-      <c r="D20" s="18" t="str">
-        <f t="shared" si="4"/>
-        <v>D20</v>
-      </c>
-      <c r="E20" s="18" t="str">
-        <f t="shared" si="4"/>
-        <v>E20</v>
-      </c>
+      <c r="B20" s="18"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="18"/>
       <c r="F20" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="G20" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>G20</v>
-      </c>
-      <c r="H20" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>H20</v>
-      </c>
-      <c r="I20" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>I20</v>
-      </c>
-      <c r="J20" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v>J20</v>
-      </c>
+      <c r="G20" s="18"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="18"/>
+      <c r="J20" s="18"/>
     </row>
     <row r="21" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="18" t="str">
-        <f t="shared" ref="B21:B24" si="5">ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>B21</v>
-      </c>
-      <c r="C21" s="18" t="str">
-        <f t="shared" si="4"/>
-        <v>C21</v>
-      </c>
-      <c r="D21" s="18" t="str">
-        <f t="shared" si="4"/>
-        <v>D21</v>
-      </c>
-      <c r="E21" s="18" t="str">
-        <f t="shared" si="4"/>
-        <v>E21</v>
-      </c>
+      <c r="B21" s="18"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="18"/>
       <c r="F21" s="21" t="s">
         <v>32</v>
       </c>
@@ -2809,121 +2579,49 @@
       <c r="A22" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="B22" s="18" t="str">
-        <f t="shared" si="5"/>
-        <v>B22</v>
-      </c>
-      <c r="C22" s="18" t="str">
-        <f t="shared" si="4"/>
-        <v>C22</v>
-      </c>
-      <c r="D22" s="18" t="str">
-        <f t="shared" si="4"/>
-        <v>D22</v>
-      </c>
-      <c r="E22" s="18" t="str">
-        <f t="shared" si="4"/>
-        <v>E22</v>
-      </c>
+      <c r="B22" s="18"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="18"/>
+      <c r="E22" s="18"/>
       <c r="F22" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="G22" s="18" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>G22</v>
-      </c>
-      <c r="H22" s="18" t="str">
-        <f t="shared" ref="H22:J22" si="6">ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>H22</v>
-      </c>
-      <c r="I22" s="18" t="str">
-        <f t="shared" si="6"/>
-        <v>I22</v>
-      </c>
-      <c r="J22" s="18" t="str">
-        <f t="shared" si="6"/>
-        <v>J22</v>
-      </c>
+      <c r="G22" s="18"/>
+      <c r="H22" s="18"/>
+      <c r="I22" s="18"/>
+      <c r="J22" s="18"/>
     </row>
     <row r="23" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="B23" s="18" t="str">
-        <f t="shared" si="5"/>
-        <v>B23</v>
-      </c>
-      <c r="C23" s="18" t="str">
-        <f t="shared" si="4"/>
-        <v>C23</v>
-      </c>
-      <c r="D23" s="18" t="str">
-        <f t="shared" si="4"/>
-        <v>D23</v>
-      </c>
-      <c r="E23" s="18" t="str">
-        <f t="shared" si="4"/>
-        <v>E23</v>
-      </c>
+      <c r="B23" s="18"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="18"/>
       <c r="F23" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="G23" s="18" t="str">
-        <f t="shared" ref="G23:J28" si="7">ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>G23</v>
-      </c>
-      <c r="H23" s="18" t="str">
-        <f t="shared" si="7"/>
-        <v>H23</v>
-      </c>
-      <c r="I23" s="18" t="str">
-        <f t="shared" si="7"/>
-        <v>I23</v>
-      </c>
-      <c r="J23" s="18" t="str">
-        <f t="shared" si="7"/>
-        <v>J23</v>
-      </c>
+      <c r="G23" s="18"/>
+      <c r="H23" s="18"/>
+      <c r="I23" s="18"/>
+      <c r="J23" s="18"/>
     </row>
     <row r="24" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="B24" s="18" t="str">
-        <f t="shared" si="5"/>
-        <v>B24</v>
-      </c>
-      <c r="C24" s="18" t="str">
-        <f t="shared" si="4"/>
-        <v>C24</v>
-      </c>
-      <c r="D24" s="18" t="str">
-        <f t="shared" si="4"/>
-        <v>D24</v>
-      </c>
-      <c r="E24" s="18" t="str">
-        <f t="shared" si="4"/>
-        <v>E24</v>
-      </c>
+      <c r="B24" s="18"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="18"/>
       <c r="F24" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="G24" s="18" t="str">
-        <f t="shared" si="7"/>
-        <v>G24</v>
-      </c>
-      <c r="H24" s="18" t="str">
-        <f t="shared" si="7"/>
-        <v>H24</v>
-      </c>
-      <c r="I24" s="18" t="str">
-        <f t="shared" si="7"/>
-        <v>I24</v>
-      </c>
-      <c r="J24" s="18" t="str">
-        <f t="shared" si="7"/>
-        <v>J24</v>
-      </c>
+      <c r="G24" s="18"/>
+      <c r="H24" s="18"/>
+      <c r="I24" s="18"/>
+      <c r="J24" s="18"/>
     </row>
     <row r="25" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="14" t="s">
@@ -2944,163 +2642,67 @@
       <c r="F25" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="G25" s="18" t="str">
-        <f t="shared" si="7"/>
-        <v>G25</v>
-      </c>
-      <c r="H25" s="18" t="str">
-        <f t="shared" si="7"/>
-        <v>H25</v>
-      </c>
-      <c r="I25" s="18" t="str">
-        <f t="shared" si="7"/>
-        <v>I25</v>
-      </c>
-      <c r="J25" s="18" t="str">
-        <f t="shared" si="7"/>
-        <v>J25</v>
-      </c>
+      <c r="G25" s="18"/>
+      <c r="H25" s="18"/>
+      <c r="I25" s="18"/>
+      <c r="J25" s="18"/>
     </row>
     <row r="26" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="B26" s="18" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>B26</v>
-      </c>
-      <c r="C26" s="18" t="str">
-        <f t="shared" ref="C26:E29" si="8">ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>C26</v>
-      </c>
-      <c r="D26" s="18" t="str">
-        <f t="shared" si="8"/>
-        <v>D26</v>
-      </c>
-      <c r="E26" s="18" t="str">
-        <f t="shared" si="8"/>
-        <v>E26</v>
-      </c>
+      <c r="B26" s="18"/>
+      <c r="C26" s="18"/>
+      <c r="D26" s="18"/>
+      <c r="E26" s="18"/>
       <c r="F26" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="G26" s="18" t="str">
-        <f t="shared" si="7"/>
-        <v>G26</v>
-      </c>
-      <c r="H26" s="18" t="str">
-        <f t="shared" si="7"/>
-        <v>H26</v>
-      </c>
-      <c r="I26" s="18" t="str">
-        <f t="shared" si="7"/>
-        <v>I26</v>
-      </c>
-      <c r="J26" s="18" t="str">
-        <f t="shared" si="7"/>
-        <v>J26</v>
-      </c>
+      <c r="G26" s="18"/>
+      <c r="H26" s="18"/>
+      <c r="I26" s="18"/>
+      <c r="J26" s="18"/>
     </row>
     <row r="27" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="B27" s="18" t="str">
-        <f t="shared" ref="B27:B29" si="9">ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>B27</v>
-      </c>
-      <c r="C27" s="18" t="str">
-        <f t="shared" si="8"/>
-        <v>C27</v>
-      </c>
-      <c r="D27" s="18" t="str">
-        <f t="shared" si="8"/>
-        <v>D27</v>
-      </c>
-      <c r="E27" s="18" t="str">
-        <f t="shared" si="8"/>
-        <v>E27</v>
-      </c>
+      <c r="B27" s="18"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="18"/>
+      <c r="E27" s="18"/>
       <c r="F27" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="G27" s="18" t="str">
-        <f t="shared" si="7"/>
-        <v>G27</v>
-      </c>
-      <c r="H27" s="18" t="str">
-        <f t="shared" si="7"/>
-        <v>H27</v>
-      </c>
-      <c r="I27" s="18" t="str">
-        <f t="shared" si="7"/>
-        <v>I27</v>
-      </c>
-      <c r="J27" s="18" t="str">
-        <f t="shared" si="7"/>
-        <v>J27</v>
-      </c>
+      <c r="G27" s="18"/>
+      <c r="H27" s="18"/>
+      <c r="I27" s="18"/>
+      <c r="J27" s="18"/>
     </row>
     <row r="28" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="B28" s="18" t="str">
-        <f t="shared" si="9"/>
-        <v>B28</v>
-      </c>
-      <c r="C28" s="18" t="str">
-        <f t="shared" si="8"/>
-        <v>C28</v>
-      </c>
-      <c r="D28" s="18" t="str">
-        <f t="shared" si="8"/>
-        <v>D28</v>
-      </c>
-      <c r="E28" s="18" t="str">
-        <f t="shared" si="8"/>
-        <v>E28</v>
-      </c>
+      <c r="B28" s="18"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="18"/>
+      <c r="E28" s="18"/>
       <c r="F28" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="G28" s="18" t="str">
-        <f t="shared" si="7"/>
-        <v>G28</v>
-      </c>
-      <c r="H28" s="18" t="str">
-        <f t="shared" si="7"/>
-        <v>H28</v>
-      </c>
-      <c r="I28" s="18" t="str">
-        <f t="shared" si="7"/>
-        <v>I28</v>
-      </c>
-      <c r="J28" s="18" t="str">
-        <f t="shared" si="7"/>
-        <v>J28</v>
-      </c>
+      <c r="G28" s="18"/>
+      <c r="H28" s="18"/>
+      <c r="I28" s="18"/>
+      <c r="J28" s="18"/>
     </row>
     <row r="29" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="B29" s="18" t="str">
-        <f t="shared" si="9"/>
-        <v>B29</v>
-      </c>
-      <c r="C29" s="18" t="str">
-        <f t="shared" si="8"/>
-        <v>C29</v>
-      </c>
-      <c r="D29" s="18" t="str">
-        <f t="shared" si="8"/>
-        <v>D29</v>
-      </c>
-      <c r="E29" s="18" t="str">
-        <f t="shared" si="8"/>
-        <v>E29</v>
-      </c>
+      <c r="B29" s="18"/>
+      <c r="C29" s="18"/>
+      <c r="D29" s="18"/>
+      <c r="E29" s="18"/>
       <c r="F29" s="15" t="s">
         <v>75</v>
       </c>
@@ -3136,83 +2738,35 @@
       <c r="F30" s="17" t="s">
         <v>76</v>
       </c>
-      <c r="G30" s="18" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>G30</v>
-      </c>
-      <c r="H30" s="18" t="str">
-        <f t="shared" ref="H30:J31" si="10">ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>H30</v>
-      </c>
-      <c r="I30" s="18" t="str">
-        <f t="shared" si="10"/>
-        <v>I30</v>
-      </c>
-      <c r="J30" s="18" t="str">
-        <f t="shared" si="10"/>
-        <v>J30</v>
-      </c>
+      <c r="G30" s="18"/>
+      <c r="H30" s="18"/>
+      <c r="I30" s="18"/>
+      <c r="J30" s="18"/>
     </row>
     <row r="31" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="B31" s="18" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>B31</v>
-      </c>
-      <c r="C31" s="18" t="str">
-        <f t="shared" ref="C31:E38" si="11">ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>C31</v>
-      </c>
-      <c r="D31" s="18" t="str">
-        <f t="shared" si="11"/>
-        <v>D31</v>
-      </c>
-      <c r="E31" s="18" t="str">
-        <f t="shared" si="11"/>
-        <v>E31</v>
-      </c>
+      <c r="B31" s="18"/>
+      <c r="C31" s="18"/>
+      <c r="D31" s="18"/>
+      <c r="E31" s="18"/>
       <c r="F31" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="G31" s="18" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>G31</v>
-      </c>
-      <c r="H31" s="18" t="str">
-        <f t="shared" si="10"/>
-        <v>H31</v>
-      </c>
-      <c r="I31" s="18" t="str">
-        <f t="shared" si="10"/>
-        <v>I31</v>
-      </c>
-      <c r="J31" s="18" t="str">
-        <f t="shared" si="10"/>
-        <v>J31</v>
-      </c>
+      <c r="G31" s="18"/>
+      <c r="H31" s="18"/>
+      <c r="I31" s="18"/>
+      <c r="J31" s="18"/>
     </row>
     <row r="32" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="17" t="s">
         <v>97</v>
       </c>
-      <c r="B32" s="18" t="str">
-        <f t="shared" ref="B32:B38" si="12">ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>B32</v>
-      </c>
-      <c r="C32" s="18" t="str">
-        <f t="shared" si="11"/>
-        <v>C32</v>
-      </c>
-      <c r="D32" s="18" t="str">
-        <f t="shared" si="11"/>
-        <v>D32</v>
-      </c>
-      <c r="E32" s="18" t="str">
-        <f t="shared" si="11"/>
-        <v>E32</v>
-      </c>
+      <c r="B32" s="18"/>
+      <c r="C32" s="18"/>
+      <c r="D32" s="18"/>
+      <c r="E32" s="18"/>
       <c r="F32" s="15" t="s">
         <v>41</v>
       </c>
@@ -3233,233 +2787,101 @@
       <c r="A33" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="B33" s="18" t="str">
-        <f t="shared" si="12"/>
-        <v>B33</v>
-      </c>
-      <c r="C33" s="18" t="str">
-        <f t="shared" si="11"/>
-        <v>C33</v>
-      </c>
-      <c r="D33" s="18" t="str">
-        <f t="shared" si="11"/>
-        <v>D33</v>
-      </c>
-      <c r="E33" s="18" t="str">
-        <f t="shared" si="11"/>
-        <v>E33</v>
-      </c>
+      <c r="B33" s="18"/>
+      <c r="C33" s="18"/>
+      <c r="D33" s="18"/>
+      <c r="E33" s="18"/>
       <c r="F33" s="17" t="s">
         <v>100</v>
       </c>
-      <c r="G33" s="18" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>G33</v>
-      </c>
-      <c r="H33" s="18" t="str">
-        <f t="shared" ref="H33:J37" si="13">ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>H33</v>
-      </c>
-      <c r="I33" s="18" t="str">
-        <f t="shared" si="13"/>
-        <v>I33</v>
-      </c>
-      <c r="J33" s="18" t="str">
-        <f t="shared" si="13"/>
-        <v>J33</v>
-      </c>
+      <c r="G33" s="18"/>
+      <c r="H33" s="18"/>
+      <c r="I33" s="18"/>
+      <c r="J33" s="18"/>
     </row>
     <row r="34" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="B34" s="18" t="str">
-        <f t="shared" si="12"/>
-        <v>B34</v>
-      </c>
-      <c r="C34" s="18" t="str">
-        <f t="shared" si="11"/>
-        <v>C34</v>
-      </c>
-      <c r="D34" s="18" t="str">
-        <f t="shared" si="11"/>
-        <v>D34</v>
-      </c>
-      <c r="E34" s="18" t="str">
-        <f t="shared" si="11"/>
-        <v>E34</v>
-      </c>
+      <c r="B34" s="18"/>
+      <c r="C34" s="18"/>
+      <c r="D34" s="18"/>
+      <c r="E34" s="18"/>
       <c r="F34" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="G34" s="18" t="str">
-        <f t="shared" ref="G34:G37" si="14">ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>G34</v>
-      </c>
-      <c r="H34" s="18" t="str">
-        <f t="shared" si="13"/>
-        <v>H34</v>
-      </c>
-      <c r="I34" s="18" t="str">
-        <f t="shared" si="13"/>
-        <v>I34</v>
-      </c>
-      <c r="J34" s="18" t="str">
-        <f t="shared" si="13"/>
-        <v>J34</v>
-      </c>
+      <c r="G34" s="18"/>
+      <c r="H34" s="18"/>
+      <c r="I34" s="18"/>
+      <c r="J34" s="18"/>
     </row>
     <row r="35" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="B35" s="18" t="str">
-        <f t="shared" si="12"/>
-        <v>B35</v>
-      </c>
-      <c r="C35" s="18" t="str">
-        <f t="shared" si="11"/>
-        <v>C35</v>
-      </c>
-      <c r="D35" s="18" t="str">
-        <f t="shared" si="11"/>
-        <v>D35</v>
-      </c>
-      <c r="E35" s="18" t="str">
-        <f t="shared" si="11"/>
-        <v>E35</v>
-      </c>
+      <c r="B35" s="18"/>
+      <c r="C35" s="18"/>
+      <c r="D35" s="18"/>
+      <c r="E35" s="18"/>
       <c r="F35" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="G35" s="18" t="str">
-        <f t="shared" si="14"/>
-        <v>G35</v>
-      </c>
-      <c r="H35" s="18" t="str">
-        <f t="shared" si="13"/>
-        <v>H35</v>
-      </c>
-      <c r="I35" s="18" t="str">
-        <f t="shared" si="13"/>
-        <v>I35</v>
-      </c>
-      <c r="J35" s="18" t="str">
-        <f t="shared" si="13"/>
-        <v>J35</v>
-      </c>
+      <c r="G35" s="18"/>
+      <c r="H35" s="18"/>
+      <c r="I35" s="18"/>
+      <c r="J35" s="18"/>
     </row>
     <row r="36" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="B36" s="18" t="str">
-        <f t="shared" si="12"/>
-        <v>B36</v>
-      </c>
-      <c r="C36" s="18" t="str">
-        <f t="shared" si="11"/>
-        <v>C36</v>
-      </c>
-      <c r="D36" s="18" t="str">
-        <f t="shared" si="11"/>
-        <v>D36</v>
-      </c>
-      <c r="E36" s="18" t="str">
-        <f t="shared" si="11"/>
-        <v>E36</v>
-      </c>
+      <c r="B36" s="18"/>
+      <c r="C36" s="18"/>
+      <c r="D36" s="18"/>
+      <c r="E36" s="18"/>
       <c r="F36" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="G36" s="18" t="str">
-        <f t="shared" si="14"/>
-        <v>G36</v>
-      </c>
-      <c r="H36" s="18" t="str">
-        <f t="shared" si="13"/>
-        <v>H36</v>
-      </c>
-      <c r="I36" s="18" t="str">
-        <f t="shared" si="13"/>
-        <v>I36</v>
-      </c>
-      <c r="J36" s="18" t="str">
-        <f t="shared" si="13"/>
-        <v>J36</v>
-      </c>
+      <c r="G36" s="18"/>
+      <c r="H36" s="18"/>
+      <c r="I36" s="18"/>
+      <c r="J36" s="18"/>
     </row>
     <row r="37" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="24" t="s">
         <v>74</v>
       </c>
-      <c r="B37" s="18" t="str">
-        <f t="shared" si="12"/>
-        <v>B37</v>
-      </c>
-      <c r="C37" s="18" t="str">
-        <f t="shared" si="11"/>
-        <v>C37</v>
-      </c>
-      <c r="D37" s="18" t="str">
-        <f t="shared" si="11"/>
-        <v>D37</v>
-      </c>
-      <c r="E37" s="18" t="str">
-        <f t="shared" si="11"/>
-        <v>E37</v>
-      </c>
+      <c r="B37" s="18"/>
+      <c r="C37" s="18"/>
+      <c r="D37" s="18"/>
+      <c r="E37" s="18"/>
       <c r="F37" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="G37" s="18" t="str">
-        <f t="shared" si="14"/>
-        <v>G37</v>
-      </c>
-      <c r="H37" s="18" t="str">
-        <f t="shared" si="13"/>
-        <v>H37</v>
-      </c>
-      <c r="I37" s="18" t="str">
-        <f t="shared" si="13"/>
-        <v>I37</v>
-      </c>
-      <c r="J37" s="18" t="str">
-        <f t="shared" si="13"/>
-        <v>J37</v>
-      </c>
+      <c r="G37" s="18"/>
+      <c r="H37" s="18"/>
+      <c r="I37" s="18"/>
+      <c r="J37" s="18"/>
     </row>
     <row r="38" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="B38" s="18" t="str">
-        <f t="shared" si="12"/>
-        <v>B38</v>
-      </c>
-      <c r="C38" s="18" t="str">
-        <f t="shared" si="11"/>
-        <v>C38</v>
-      </c>
-      <c r="D38" s="18" t="str">
-        <f t="shared" si="11"/>
-        <v>D38</v>
-      </c>
-      <c r="E38" s="18" t="str">
-        <f t="shared" si="11"/>
-        <v>E38</v>
-      </c>
+      <c r="B38" s="18"/>
+      <c r="C38" s="18"/>
+      <c r="D38" s="18"/>
+      <c r="E38" s="18"/>
       <c r="F38" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="G38" s="42" t="s">
+      <c r="G38" s="71" t="s">
         <v>90</v>
       </c>
-      <c r="H38" s="43"/>
-      <c r="I38" s="44" t="s">
+      <c r="H38" s="72"/>
+      <c r="I38" s="73" t="s">
         <v>91</v>
       </c>
-      <c r="J38" s="45"/>
+      <c r="J38" s="74"/>
     </row>
     <row r="39" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="14" t="s">
@@ -3480,345 +2902,309 @@
       <c r="F39" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="G39" s="27" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>G39</v>
-      </c>
+      <c r="G39" s="27"/>
       <c r="H39" s="28"/>
-      <c r="I39" s="27" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>I39</v>
-      </c>
+      <c r="I39" s="27"/>
       <c r="J39" s="28"/>
     </row>
     <row r="40" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="B40" s="18" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>B40</v>
-      </c>
-      <c r="C40" s="18" t="str">
-        <f t="shared" ref="C40:E43" si="15">ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>C40</v>
-      </c>
-      <c r="D40" s="18" t="str">
-        <f t="shared" si="15"/>
-        <v>D40</v>
-      </c>
-      <c r="E40" s="18" t="str">
-        <f t="shared" si="15"/>
-        <v>E40</v>
-      </c>
+      <c r="B40" s="18"/>
+      <c r="C40" s="18"/>
+      <c r="D40" s="18"/>
+      <c r="E40" s="18"/>
       <c r="F40" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="G40" s="26" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>G40</v>
-      </c>
-      <c r="H40" s="26" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>H40</v>
-      </c>
-      <c r="I40" s="18" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>I40</v>
-      </c>
-      <c r="J40" s="26" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>J40</v>
-      </c>
+      <c r="G40" s="26"/>
+      <c r="H40" s="26"/>
+      <c r="I40" s="18"/>
+      <c r="J40" s="26"/>
     </row>
     <row r="41" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="B41" s="18" t="str">
-        <f t="shared" ref="B41:B43" si="16">ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>B41</v>
-      </c>
-      <c r="C41" s="18" t="str">
-        <f t="shared" si="15"/>
-        <v>C41</v>
-      </c>
-      <c r="D41" s="18" t="str">
-        <f t="shared" si="15"/>
-        <v>D41</v>
-      </c>
-      <c r="E41" s="18" t="str">
-        <f t="shared" si="15"/>
-        <v>E41</v>
-      </c>
+      <c r="B41" s="18"/>
+      <c r="C41" s="18"/>
+      <c r="D41" s="18"/>
+      <c r="E41" s="18"/>
       <c r="F41" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="G41" s="64" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>G41</v>
-      </c>
-      <c r="H41" s="65"/>
-      <c r="I41" s="64" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>I41</v>
-      </c>
-      <c r="J41" s="65"/>
+      <c r="G41" s="33"/>
+      <c r="H41" s="34"/>
+      <c r="I41" s="33"/>
+      <c r="J41" s="34"/>
     </row>
     <row r="42" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="B42" s="18" t="str">
-        <f t="shared" si="16"/>
-        <v>B42</v>
-      </c>
-      <c r="C42" s="18" t="str">
-        <f t="shared" si="15"/>
-        <v>C42</v>
-      </c>
-      <c r="D42" s="18" t="str">
-        <f t="shared" si="15"/>
-        <v>D42</v>
-      </c>
-      <c r="E42" s="18" t="str">
-        <f t="shared" si="15"/>
-        <v>E42</v>
-      </c>
+      <c r="B42" s="18"/>
+      <c r="C42" s="18"/>
+      <c r="D42" s="18"/>
+      <c r="E42" s="18"/>
       <c r="F42" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="G42" s="64" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>G42</v>
-      </c>
-      <c r="H42" s="65"/>
-      <c r="I42" s="64" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>I42</v>
-      </c>
-      <c r="J42" s="65"/>
+      <c r="G42" s="33"/>
+      <c r="H42" s="34"/>
+      <c r="I42" s="33"/>
+      <c r="J42" s="34"/>
     </row>
     <row r="43" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="B43" s="18" t="str">
-        <f t="shared" si="16"/>
-        <v>B43</v>
-      </c>
-      <c r="C43" s="18" t="str">
-        <f t="shared" si="15"/>
-        <v>C43</v>
-      </c>
-      <c r="D43" s="18" t="str">
-        <f t="shared" si="15"/>
-        <v>D43</v>
-      </c>
-      <c r="E43" s="18" t="str">
-        <f t="shared" si="15"/>
-        <v>E43</v>
-      </c>
+      <c r="B43" s="18"/>
+      <c r="C43" s="18"/>
+      <c r="D43" s="18"/>
+      <c r="E43" s="18"/>
       <c r="F43" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="G43" s="64" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>G43</v>
-      </c>
-      <c r="H43" s="65"/>
-      <c r="I43" s="64" t="str">
-        <f>ADDRESS(ROW(),COLUMN(),4)</f>
-        <v>I43</v>
-      </c>
-      <c r="J43" s="65"/>
+      <c r="G43" s="33"/>
+      <c r="H43" s="34"/>
+      <c r="I43" s="33"/>
+      <c r="J43" s="34"/>
     </row>
     <row r="44" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="46" t="s">
+      <c r="A44" s="65" t="s">
         <v>61</v>
       </c>
-      <c r="B44" s="50"/>
-      <c r="C44" s="50"/>
-      <c r="D44" s="50"/>
-      <c r="E44" s="50"/>
-      <c r="F44" s="50"/>
-      <c r="G44" s="50"/>
-      <c r="H44" s="50"/>
-      <c r="I44" s="50"/>
-      <c r="J44" s="54"/>
+      <c r="B44" s="69"/>
+      <c r="C44" s="69"/>
+      <c r="D44" s="69"/>
+      <c r="E44" s="69"/>
+      <c r="F44" s="69"/>
+      <c r="G44" s="69"/>
+      <c r="H44" s="69"/>
+      <c r="I44" s="69"/>
+      <c r="J44" s="70"/>
     </row>
     <row r="45" spans="1:10" s="2" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="46" t="s">
+      <c r="A45" s="65" t="s">
         <v>62</v>
       </c>
-      <c r="B45" s="47"/>
-      <c r="C45" s="48"/>
-      <c r="D45" s="49" t="s">
+      <c r="B45" s="66"/>
+      <c r="C45" s="67"/>
+      <c r="D45" s="68" t="s">
         <v>59</v>
       </c>
-      <c r="E45" s="47"/>
-      <c r="F45" s="48"/>
-      <c r="G45" s="50" t="s">
+      <c r="E45" s="66"/>
+      <c r="F45" s="67"/>
+      <c r="G45" s="69" t="s">
         <v>63</v>
       </c>
-      <c r="H45" s="47"/>
-      <c r="I45" s="47"/>
-      <c r="J45" s="48"/>
+      <c r="H45" s="66"/>
+      <c r="I45" s="66"/>
+      <c r="J45" s="67"/>
     </row>
     <row r="46" spans="1:10" s="2" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="66" t="s">
+      <c r="A46" s="47" t="s">
         <v>77</v>
       </c>
-      <c r="B46" s="67"/>
-      <c r="C46" s="68"/>
-      <c r="D46" s="72" t="s">
+      <c r="B46" s="48"/>
+      <c r="C46" s="49"/>
+      <c r="D46" s="62" t="s">
         <v>64</v>
       </c>
-      <c r="E46" s="73"/>
-      <c r="F46" s="74"/>
-      <c r="G46" s="66" t="s">
+      <c r="E46" s="63"/>
+      <c r="F46" s="64"/>
+      <c r="G46" s="47" t="s">
         <v>105</v>
       </c>
-      <c r="H46" s="67"/>
-      <c r="I46" s="67"/>
-      <c r="J46" s="68"/>
+      <c r="H46" s="48"/>
+      <c r="I46" s="48"/>
+      <c r="J46" s="49"/>
     </row>
     <row r="47" spans="1:10" s="2" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="55" t="s">
+      <c r="A47" s="50" t="s">
         <v>78</v>
       </c>
-      <c r="B47" s="56"/>
-      <c r="C47" s="57"/>
-      <c r="D47" s="51" t="s">
+      <c r="B47" s="51"/>
+      <c r="C47" s="52"/>
+      <c r="D47" s="41" t="s">
         <v>65</v>
       </c>
-      <c r="E47" s="52"/>
-      <c r="F47" s="53"/>
-      <c r="G47" s="55" t="s">
+      <c r="E47" s="42"/>
+      <c r="F47" s="43"/>
+      <c r="G47" s="50" t="s">
         <v>106</v>
       </c>
-      <c r="H47" s="56"/>
-      <c r="I47" s="56"/>
-      <c r="J47" s="57"/>
+      <c r="H47" s="51"/>
+      <c r="I47" s="51"/>
+      <c r="J47" s="52"/>
     </row>
     <row r="48" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="55" t="s">
+      <c r="A48" s="50" t="s">
         <v>79</v>
       </c>
-      <c r="B48" s="56"/>
-      <c r="C48" s="57"/>
-      <c r="D48" s="51" t="s">
+      <c r="B48" s="51"/>
+      <c r="C48" s="52"/>
+      <c r="D48" s="41" t="s">
         <v>66</v>
       </c>
-      <c r="E48" s="52"/>
-      <c r="F48" s="53"/>
-      <c r="G48" s="55"/>
-      <c r="H48" s="56"/>
-      <c r="I48" s="56"/>
-      <c r="J48" s="57"/>
+      <c r="E48" s="42"/>
+      <c r="F48" s="43"/>
+      <c r="G48" s="50"/>
+      <c r="H48" s="51"/>
+      <c r="I48" s="51"/>
+      <c r="J48" s="52"/>
     </row>
     <row r="49" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="55" t="s">
+      <c r="A49" s="50" t="s">
         <v>82</v>
       </c>
-      <c r="B49" s="56"/>
-      <c r="C49" s="57"/>
-      <c r="D49" s="51" t="s">
+      <c r="B49" s="51"/>
+      <c r="C49" s="52"/>
+      <c r="D49" s="41" t="s">
         <v>67</v>
       </c>
-      <c r="E49" s="52"/>
-      <c r="F49" s="53"/>
-      <c r="G49" s="55"/>
-      <c r="H49" s="56"/>
-      <c r="I49" s="56"/>
-      <c r="J49" s="57"/>
+      <c r="E49" s="42"/>
+      <c r="F49" s="43"/>
+      <c r="G49" s="50"/>
+      <c r="H49" s="51"/>
+      <c r="I49" s="51"/>
+      <c r="J49" s="52"/>
     </row>
     <row r="50" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="55" t="s">
+      <c r="A50" s="50" t="s">
         <v>80</v>
       </c>
-      <c r="B50" s="56"/>
-      <c r="C50" s="57"/>
-      <c r="D50" s="51" t="s">
+      <c r="B50" s="51"/>
+      <c r="C50" s="52"/>
+      <c r="D50" s="41" t="s">
         <v>68</v>
       </c>
-      <c r="E50" s="52"/>
-      <c r="F50" s="53"/>
-      <c r="G50" s="58"/>
-      <c r="H50" s="59"/>
-      <c r="I50" s="59"/>
-      <c r="J50" s="60"/>
+      <c r="E50" s="42"/>
+      <c r="F50" s="43"/>
+      <c r="G50" s="53"/>
+      <c r="H50" s="54"/>
+      <c r="I50" s="54"/>
+      <c r="J50" s="55"/>
     </row>
     <row r="51" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="69" t="s">
+      <c r="A51" s="59" t="s">
         <v>81</v>
       </c>
-      <c r="B51" s="70"/>
-      <c r="C51" s="71"/>
-      <c r="D51" s="84" t="s">
+      <c r="B51" s="60"/>
+      <c r="C51" s="61"/>
+      <c r="D51" s="44" t="s">
         <v>69</v>
       </c>
-      <c r="E51" s="85"/>
-      <c r="F51" s="86"/>
-      <c r="G51" s="61" t="s">
+      <c r="E51" s="45"/>
+      <c r="F51" s="46"/>
+      <c r="G51" s="56" t="s">
         <v>83</v>
       </c>
-      <c r="H51" s="62"/>
-      <c r="I51" s="62"/>
-      <c r="J51" s="63"/>
+      <c r="H51" s="57"/>
+      <c r="I51" s="57"/>
+      <c r="J51" s="58"/>
     </row>
     <row r="52" spans="1:10" ht="18" x14ac:dyDescent="0.3">
       <c r="A52" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="B52" s="78"/>
-      <c r="C52" s="79"/>
-      <c r="D52" s="79"/>
-      <c r="E52" s="79"/>
-      <c r="F52" s="79"/>
-      <c r="G52" s="79"/>
-      <c r="H52" s="79"/>
-      <c r="I52" s="79"/>
-      <c r="J52" s="80"/>
+      <c r="B52" s="35"/>
+      <c r="C52" s="36"/>
+      <c r="D52" s="36"/>
+      <c r="E52" s="36"/>
+      <c r="F52" s="36"/>
+      <c r="G52" s="36"/>
+      <c r="H52" s="36"/>
+      <c r="I52" s="36"/>
+      <c r="J52" s="37"/>
     </row>
     <row r="53" spans="1:10" ht="18" x14ac:dyDescent="0.3">
-      <c r="A53" s="81"/>
-      <c r="B53" s="82"/>
-      <c r="C53" s="82"/>
-      <c r="D53" s="82"/>
-      <c r="E53" s="82"/>
-      <c r="F53" s="82"/>
-      <c r="G53" s="82"/>
-      <c r="H53" s="82"/>
-      <c r="I53" s="82"/>
-      <c r="J53" s="83"/>
+      <c r="A53" s="38"/>
+      <c r="B53" s="39"/>
+      <c r="C53" s="39"/>
+      <c r="D53" s="39"/>
+      <c r="E53" s="39"/>
+      <c r="F53" s="39"/>
+      <c r="G53" s="39"/>
+      <c r="H53" s="39"/>
+      <c r="I53" s="39"/>
+      <c r="J53" s="40"/>
     </row>
     <row r="54" spans="1:10" ht="18" x14ac:dyDescent="0.3">
-      <c r="A54" s="81"/>
-      <c r="B54" s="82"/>
-      <c r="C54" s="82"/>
-      <c r="D54" s="82"/>
-      <c r="E54" s="82"/>
-      <c r="F54" s="82"/>
-      <c r="G54" s="82"/>
-      <c r="H54" s="82"/>
-      <c r="I54" s="82"/>
-      <c r="J54" s="83"/>
+      <c r="A54" s="38"/>
+      <c r="B54" s="39"/>
+      <c r="C54" s="39"/>
+      <c r="D54" s="39"/>
+      <c r="E54" s="39"/>
+      <c r="F54" s="39"/>
+      <c r="G54" s="39"/>
+      <c r="H54" s="39"/>
+      <c r="I54" s="39"/>
+      <c r="J54" s="40"/>
     </row>
     <row r="55" spans="1:10" ht="18" x14ac:dyDescent="0.3">
-      <c r="A55" s="75"/>
-      <c r="B55" s="76"/>
-      <c r="C55" s="76"/>
-      <c r="D55" s="76"/>
-      <c r="E55" s="76"/>
-      <c r="F55" s="76"/>
-      <c r="G55" s="76"/>
-      <c r="H55" s="76"/>
-      <c r="I55" s="76"/>
-      <c r="J55" s="77"/>
+      <c r="A55" s="30"/>
+      <c r="B55" s="31"/>
+      <c r="C55" s="31"/>
+      <c r="D55" s="31"/>
+      <c r="E55" s="31"/>
+      <c r="F55" s="31"/>
+      <c r="G55" s="31"/>
+      <c r="H55" s="31"/>
+      <c r="I55" s="31"/>
+      <c r="J55" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="64">
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="D45:F45"/>
+    <mergeCell ref="G45:J45"/>
+    <mergeCell ref="D47:F47"/>
+    <mergeCell ref="A44:J44"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="I38:J38"/>
+    <mergeCell ref="G41:H41"/>
+    <mergeCell ref="I41:J41"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="I43:J43"/>
+    <mergeCell ref="G42:H42"/>
+    <mergeCell ref="I42:J42"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="G48:J48"/>
+    <mergeCell ref="G49:J49"/>
+    <mergeCell ref="G50:J50"/>
+    <mergeCell ref="G51:J51"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="A49:C49"/>
+    <mergeCell ref="A50:C50"/>
+    <mergeCell ref="A51:C51"/>
+    <mergeCell ref="D46:F46"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
     <mergeCell ref="A55:J55"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="I9:J9"/>
@@ -3835,54 +3221,6 @@
     <mergeCell ref="D51:F51"/>
     <mergeCell ref="G46:J46"/>
     <mergeCell ref="G47:J47"/>
-    <mergeCell ref="G48:J48"/>
-    <mergeCell ref="G49:J49"/>
-    <mergeCell ref="G50:J50"/>
-    <mergeCell ref="G51:J51"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="A46:C46"/>
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="A48:C48"/>
-    <mergeCell ref="A49:C49"/>
-    <mergeCell ref="A50:C50"/>
-    <mergeCell ref="A51:C51"/>
-    <mergeCell ref="D46:F46"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="A45:C45"/>
-    <mergeCell ref="D45:F45"/>
-    <mergeCell ref="G45:J45"/>
-    <mergeCell ref="D47:F47"/>
-    <mergeCell ref="A44:J44"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="I38:J38"/>
-    <mergeCell ref="G41:H41"/>
-    <mergeCell ref="I41:J41"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="I43:J43"/>
-    <mergeCell ref="G42:H42"/>
-    <mergeCell ref="I42:J42"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="I3:J3"/>
   </mergeCells>
   <dataValidations disablePrompts="1" count="1">
     <dataValidation showInputMessage="1" showErrorMessage="1" sqref="B6:F6" xr:uid="{00000000-0002-0000-0000-000000000000}"/>

</xml_diff>

<commit_message>
Update mapping and template files
</commit_message>
<xml_diff>
--- a/config/Gait Lab Physical Exam Template 2026.xlsx
+++ b/config/Gait Lab Physical Exam Template 2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://autuni-my.sharepoint.com/personal/em19830_aut_ac_nz/Documents/HRRI Gait lab/Motion Connect Databank/PyCharm/databank_export/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="57" documentId="11_8ED2F9A0AE62749DF43FEA088F4C3829D5A37722" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44ECFE8D-95DC-46C3-BCCF-23EB57E6681F}"/>
+  <xr:revisionPtr revIDLastSave="59" documentId="11_8ED2F9A0AE62749DF43FEA088F4C3829D5A37722" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C8BCC429-5BE6-4438-9D3C-1D7C5F1DE3D5}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="660" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1370,7 +1370,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1389,9 +1389,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1447,34 +1444,68 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1485,18 +1516,9 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1506,6 +1528,9 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1518,69 +1543,41 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="277">
@@ -2192,987 +2189,1003 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="A1" s="81" t="s">
+      <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="82"/>
-      <c r="C1" s="82"/>
-      <c r="D1" s="82"/>
-      <c r="E1" s="82"/>
-      <c r="F1" s="82"/>
-      <c r="G1" s="82"/>
-      <c r="H1" s="82"/>
-      <c r="I1" s="82"/>
-      <c r="J1" s="82"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
     </row>
     <row r="2" spans="1:10" ht="18" x14ac:dyDescent="0.35">
-      <c r="A2" s="83"/>
-      <c r="B2" s="83"/>
-      <c r="C2" s="83"/>
-      <c r="D2" s="83"/>
-      <c r="E2" s="83"/>
-      <c r="F2" s="83"/>
-      <c r="G2" s="83"/>
-      <c r="H2" s="83"/>
-      <c r="I2" s="83"/>
-      <c r="J2" s="83"/>
+      <c r="A2" s="35"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35"/>
     </row>
     <row r="3" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="84"/>
-      <c r="C3" s="84"/>
-      <c r="D3" s="84"/>
-      <c r="E3" s="84"/>
-      <c r="F3" s="84"/>
-      <c r="G3" s="85" t="s">
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
+      <c r="D3" s="36"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="37" t="s">
         <v>104</v>
       </c>
-      <c r="H3" s="85"/>
-      <c r="I3" s="84"/>
-      <c r="J3" s="86"/>
+      <c r="H3" s="37"/>
+      <c r="I3" s="36"/>
+      <c r="J3" s="38"/>
     </row>
     <row r="4" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B4" s="79"/>
-      <c r="C4" s="76"/>
-      <c r="D4" s="80" t="s">
+      <c r="B4" s="29"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="31" t="s">
         <v>89</v>
       </c>
-      <c r="E4" s="80"/>
+      <c r="E4" s="31"/>
       <c r="F4" s="5"/>
-      <c r="G4" s="80" t="s">
+      <c r="G4" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="H4" s="80"/>
-      <c r="I4" s="79"/>
-      <c r="J4" s="77"/>
+      <c r="H4" s="31"/>
+      <c r="I4" s="29"/>
+      <c r="J4" s="32"/>
     </row>
     <row r="5" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="75"/>
-      <c r="C5" s="76"/>
-      <c r="D5" s="76"/>
+      <c r="B5" s="39"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
       <c r="E5" s="6" t="s">
         <v>4</v>
       </c>
       <c r="F5" s="7"/>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="H5" s="8"/>
-      <c r="I5" s="76"/>
-      <c r="J5" s="77"/>
+      <c r="H5" s="31"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="32"/>
     </row>
     <row r="6" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="78"/>
-      <c r="C6" s="78"/>
-      <c r="D6" s="78"/>
-      <c r="E6" s="78"/>
-      <c r="F6" s="78"/>
-      <c r="G6" s="10" t="s">
+      <c r="B6" s="40"/>
+      <c r="C6" s="40"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="40"/>
+      <c r="F6" s="40"/>
+      <c r="G6" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="H6" s="11"/>
-      <c r="I6" s="12" t="s">
+      <c r="H6" s="10"/>
+      <c r="I6" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="J6" s="13"/>
+      <c r="J6" s="12"/>
     </row>
     <row r="7" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="71" t="s">
+      <c r="B7" s="41" t="s">
         <v>90</v>
       </c>
-      <c r="C7" s="72"/>
-      <c r="D7" s="71" t="s">
+      <c r="C7" s="42"/>
+      <c r="D7" s="41" t="s">
         <v>91</v>
       </c>
-      <c r="E7" s="72"/>
-      <c r="F7" s="15" t="s">
+      <c r="E7" s="42"/>
+      <c r="F7" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="G7" s="71" t="s">
+      <c r="G7" s="41" t="s">
         <v>90</v>
       </c>
-      <c r="H7" s="72"/>
-      <c r="I7" s="73" t="s">
+      <c r="H7" s="42"/>
+      <c r="I7" s="43" t="s">
         <v>91</v>
       </c>
-      <c r="J7" s="74"/>
+      <c r="J7" s="44"/>
     </row>
     <row r="8" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="33"/>
-      <c r="C8" s="34"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="34"/>
-      <c r="F8" s="15" t="s">
+      <c r="B8" s="45"/>
+      <c r="C8" s="46"/>
+      <c r="D8" s="45"/>
+      <c r="E8" s="46"/>
+      <c r="F8" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="33"/>
-      <c r="H8" s="34"/>
-      <c r="I8" s="33"/>
-      <c r="J8" s="34"/>
+      <c r="G8" s="45"/>
+      <c r="H8" s="46"/>
+      <c r="I8" s="45"/>
+      <c r="J8" s="46"/>
     </row>
     <row r="9" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="B9" s="33"/>
-      <c r="C9" s="34"/>
-      <c r="D9" s="33"/>
-      <c r="E9" s="34"/>
-      <c r="F9" s="17" t="s">
+      <c r="B9" s="45"/>
+      <c r="C9" s="46"/>
+      <c r="D9" s="45"/>
+      <c r="E9" s="46"/>
+      <c r="F9" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="33"/>
-      <c r="H9" s="34"/>
-      <c r="I9" s="33"/>
-      <c r="J9" s="34"/>
+      <c r="G9" s="45"/>
+      <c r="H9" s="46"/>
+      <c r="I9" s="45"/>
+      <c r="J9" s="46"/>
     </row>
     <row r="10" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="B10" s="33"/>
-      <c r="C10" s="34"/>
-      <c r="D10" s="33"/>
-      <c r="E10" s="34"/>
-      <c r="F10" s="17" t="s">
+      <c r="B10" s="45"/>
+      <c r="C10" s="46"/>
+      <c r="D10" s="45"/>
+      <c r="E10" s="46"/>
+      <c r="F10" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="G10" s="33"/>
-      <c r="H10" s="34"/>
-      <c r="I10" s="33"/>
-      <c r="J10" s="34"/>
+      <c r="G10" s="45"/>
+      <c r="H10" s="46"/>
+      <c r="I10" s="45"/>
+      <c r="J10" s="46"/>
     </row>
     <row r="11" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="B11" s="33"/>
-      <c r="C11" s="34"/>
-      <c r="D11" s="33"/>
-      <c r="E11" s="34"/>
-      <c r="F11" s="15" t="s">
+      <c r="B11" s="45"/>
+      <c r="C11" s="46"/>
+      <c r="D11" s="45"/>
+      <c r="E11" s="46"/>
+      <c r="F11" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="G11" s="19" t="s">
+      <c r="G11" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="H11" s="19" t="s">
+      <c r="H11" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="I11" s="19" t="s">
+      <c r="I11" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="J11" s="19" t="s">
+      <c r="J11" s="18" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="19" t="s">
+      <c r="C12" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="19" t="s">
+      <c r="D12" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="E12" s="19" t="s">
+      <c r="E12" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="F12" s="17" t="s">
+      <c r="F12" s="16" t="s">
         <v>99</v>
       </c>
-      <c r="G12" s="18"/>
-      <c r="H12" s="18"/>
-      <c r="I12" s="18"/>
-      <c r="J12" s="18"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
+      <c r="J12" s="17"/>
     </row>
     <row r="13" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="17" t="s">
+      <c r="A13" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="18"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="17" t="s">
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="18"/>
-      <c r="J13" s="18"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="17"/>
+      <c r="J13" s="17"/>
     </row>
     <row r="14" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="17" t="s">
+      <c r="A14" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="18"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="17" t="s">
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
-      <c r="I14" s="18"/>
-      <c r="J14" s="18"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17"/>
+      <c r="J14" s="17"/>
     </row>
     <row r="15" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="17" t="s">
+      <c r="A15" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="17" t="s">
+      <c r="B15" s="17"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="G15" s="18"/>
-      <c r="H15" s="18"/>
-      <c r="I15" s="18"/>
-      <c r="J15" s="18"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="17"/>
+      <c r="I15" s="17"/>
+      <c r="J15" s="17"/>
     </row>
     <row r="16" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="17" t="s">
+      <c r="A16" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="18"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="15" t="s">
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="G16" s="19" t="s">
+      <c r="G16" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="H16" s="19" t="s">
+      <c r="H16" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="I16" s="19" t="s">
+      <c r="I16" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="J16" s="19" t="s">
+      <c r="J16" s="18" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="17" t="s">
+      <c r="A17" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="18"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="17" t="s">
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="G17" s="18"/>
-      <c r="H17" s="18"/>
-      <c r="I17" s="18"/>
-      <c r="J17" s="18"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="17"/>
     </row>
     <row r="18" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="17" t="s">
+      <c r="A18" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="18"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="17" t="s">
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18"/>
-      <c r="I18" s="18"/>
-      <c r="J18" s="18"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="17"/>
+      <c r="I18" s="17"/>
+      <c r="J18" s="17"/>
     </row>
     <row r="19" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="19" t="s">
+      <c r="B19" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="C19" s="19" t="s">
+      <c r="C19" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="D19" s="19" t="s">
+      <c r="D19" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="E19" s="19" t="s">
+      <c r="E19" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="F19" s="17" t="s">
+      <c r="F19" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
-      <c r="I19" s="18"/>
-      <c r="J19" s="18"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="17"/>
+      <c r="I19" s="17"/>
+      <c r="J19" s="17"/>
     </row>
     <row r="20" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="17" t="s">
+      <c r="A20" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="B20" s="18"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="20" t="s">
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="G20" s="18"/>
-      <c r="H20" s="18"/>
-      <c r="I20" s="18"/>
-      <c r="J20" s="18"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="17"/>
+      <c r="I20" s="17"/>
+      <c r="J20" s="17"/>
     </row>
     <row r="21" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="17" t="s">
+      <c r="A21" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="18"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="21" t="s">
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="G21" s="29" t="s">
+      <c r="G21" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="H21" s="29" t="s">
+      <c r="H21" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="I21" s="29" t="s">
+      <c r="I21" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="J21" s="29" t="s">
+      <c r="J21" s="28" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="17" t="s">
+      <c r="A22" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="B22" s="18"/>
-      <c r="C22" s="18"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="18"/>
-      <c r="F22" s="17" t="s">
+      <c r="B22" s="17"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="G22" s="18"/>
-      <c r="H22" s="18"/>
-      <c r="I22" s="18"/>
-      <c r="J22" s="18"/>
+      <c r="G22" s="17"/>
+      <c r="H22" s="17"/>
+      <c r="I22" s="17"/>
+      <c r="J22" s="17"/>
     </row>
     <row r="23" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="17" t="s">
+      <c r="A23" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="B23" s="18"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="18"/>
-      <c r="F23" s="17" t="s">
+      <c r="B23" s="17"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="G23" s="18"/>
-      <c r="H23" s="18"/>
-      <c r="I23" s="18"/>
-      <c r="J23" s="18"/>
+      <c r="G23" s="17"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="17"/>
+      <c r="J23" s="17"/>
     </row>
     <row r="24" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="17" t="s">
+      <c r="A24" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="B24" s="18"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="18"/>
-      <c r="F24" s="17" t="s">
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="G24" s="18"/>
-      <c r="H24" s="18"/>
-      <c r="I24" s="18"/>
-      <c r="J24" s="18"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="17"/>
+      <c r="J24" s="17"/>
     </row>
     <row r="25" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="14" t="s">
+      <c r="A25" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="B25" s="19" t="s">
+      <c r="B25" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="C25" s="19" t="s">
+      <c r="C25" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="D25" s="19" t="s">
+      <c r="D25" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="E25" s="19" t="s">
+      <c r="E25" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="F25" s="17" t="s">
+      <c r="F25" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="G25" s="18"/>
-      <c r="H25" s="18"/>
-      <c r="I25" s="18"/>
-      <c r="J25" s="18"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
+      <c r="J25" s="17"/>
     </row>
     <row r="26" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="17" t="s">
+      <c r="A26" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="B26" s="18"/>
-      <c r="C26" s="18"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="17" t="s">
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="G26" s="18"/>
-      <c r="H26" s="18"/>
-      <c r="I26" s="18"/>
-      <c r="J26" s="18"/>
+      <c r="G26" s="17"/>
+      <c r="H26" s="17"/>
+      <c r="I26" s="17"/>
+      <c r="J26" s="17"/>
     </row>
     <row r="27" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="17" t="s">
+      <c r="A27" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="B27" s="18"/>
-      <c r="C27" s="18"/>
-      <c r="D27" s="18"/>
-      <c r="E27" s="18"/>
-      <c r="F27" s="17" t="s">
+      <c r="B27" s="17"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="G27" s="18"/>
-      <c r="H27" s="18"/>
-      <c r="I27" s="18"/>
-      <c r="J27" s="18"/>
+      <c r="G27" s="17"/>
+      <c r="H27" s="17"/>
+      <c r="I27" s="17"/>
+      <c r="J27" s="17"/>
     </row>
     <row r="28" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="17" t="s">
+      <c r="A28" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="B28" s="18"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
-      <c r="F28" s="22" t="s">
+      <c r="B28" s="17"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="G28" s="18"/>
-      <c r="H28" s="18"/>
-      <c r="I28" s="18"/>
-      <c r="J28" s="18"/>
+      <c r="G28" s="17"/>
+      <c r="H28" s="17"/>
+      <c r="I28" s="17"/>
+      <c r="J28" s="17"/>
     </row>
     <row r="29" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="17" t="s">
+      <c r="A29" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="B29" s="18"/>
-      <c r="C29" s="18"/>
-      <c r="D29" s="18"/>
-      <c r="E29" s="18"/>
-      <c r="F29" s="15" t="s">
+      <c r="B29" s="17"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="G29" s="29" t="s">
+      <c r="G29" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="H29" s="29" t="s">
+      <c r="H29" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="I29" s="29" t="s">
+      <c r="I29" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="J29" s="29" t="s">
+      <c r="J29" s="28" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="30" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="14" t="s">
+      <c r="A30" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="B30" s="19" t="s">
+      <c r="B30" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="C30" s="19" t="s">
+      <c r="C30" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="D30" s="19" t="s">
+      <c r="D30" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="E30" s="19" t="s">
+      <c r="E30" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="F30" s="17" t="s">
+      <c r="F30" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="G30" s="18"/>
-      <c r="H30" s="18"/>
-      <c r="I30" s="18"/>
-      <c r="J30" s="18"/>
+      <c r="G30" s="17"/>
+      <c r="H30" s="17"/>
+      <c r="I30" s="17"/>
+      <c r="J30" s="17"/>
     </row>
     <row r="31" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="17" t="s">
+      <c r="A31" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="B31" s="18"/>
-      <c r="C31" s="18"/>
-      <c r="D31" s="18"/>
-      <c r="E31" s="18"/>
-      <c r="F31" s="17" t="s">
+      <c r="B31" s="17"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17"/>
+      <c r="F31" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="G31" s="18"/>
-      <c r="H31" s="18"/>
-      <c r="I31" s="18"/>
-      <c r="J31" s="18"/>
+      <c r="G31" s="17"/>
+      <c r="H31" s="17"/>
+      <c r="I31" s="17"/>
+      <c r="J31" s="17"/>
     </row>
     <row r="32" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="17" t="s">
+      <c r="A32" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="B32" s="18"/>
-      <c r="C32" s="18"/>
-      <c r="D32" s="18"/>
-      <c r="E32" s="18"/>
-      <c r="F32" s="15" t="s">
+      <c r="B32" s="17"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="G32" s="29" t="s">
+      <c r="G32" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="H32" s="29" t="s">
+      <c r="H32" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="I32" s="29" t="s">
+      <c r="I32" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="J32" s="29" t="s">
+      <c r="J32" s="28" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="33" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="17" t="s">
+      <c r="A33" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="B33" s="18"/>
-      <c r="C33" s="18"/>
-      <c r="D33" s="18"/>
-      <c r="E33" s="18"/>
-      <c r="F33" s="17" t="s">
+      <c r="B33" s="17"/>
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="G33" s="18"/>
-      <c r="H33" s="18"/>
-      <c r="I33" s="18"/>
-      <c r="J33" s="18"/>
+      <c r="G33" s="17"/>
+      <c r="H33" s="17"/>
+      <c r="I33" s="17"/>
+      <c r="J33" s="17"/>
     </row>
     <row r="34" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="17" t="s">
+      <c r="A34" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="B34" s="18"/>
-      <c r="C34" s="18"/>
-      <c r="D34" s="18"/>
-      <c r="E34" s="18"/>
-      <c r="F34" s="17" t="s">
+      <c r="B34" s="17"/>
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
+      <c r="F34" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="G34" s="18"/>
-      <c r="H34" s="18"/>
-      <c r="I34" s="18"/>
-      <c r="J34" s="18"/>
+      <c r="G34" s="17"/>
+      <c r="H34" s="17"/>
+      <c r="I34" s="17"/>
+      <c r="J34" s="17"/>
     </row>
     <row r="35" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="17" t="s">
+      <c r="A35" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="B35" s="18"/>
-      <c r="C35" s="18"/>
-      <c r="D35" s="18"/>
-      <c r="E35" s="18"/>
-      <c r="F35" s="17" t="s">
+      <c r="B35" s="17"/>
+      <c r="C35" s="17"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="17"/>
+      <c r="F35" s="16" t="s">
         <v>102</v>
       </c>
-      <c r="G35" s="18"/>
-      <c r="H35" s="18"/>
-      <c r="I35" s="18"/>
-      <c r="J35" s="18"/>
+      <c r="G35" s="17"/>
+      <c r="H35" s="17"/>
+      <c r="I35" s="17"/>
+      <c r="J35" s="17"/>
     </row>
     <row r="36" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="17" t="s">
+      <c r="A36" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="B36" s="18"/>
-      <c r="C36" s="18"/>
-      <c r="D36" s="18"/>
-      <c r="E36" s="18"/>
-      <c r="F36" s="17" t="s">
+      <c r="B36" s="17"/>
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="17"/>
+      <c r="F36" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="G36" s="18"/>
-      <c r="H36" s="18"/>
-      <c r="I36" s="18"/>
-      <c r="J36" s="18"/>
+      <c r="G36" s="17"/>
+      <c r="H36" s="17"/>
+      <c r="I36" s="17"/>
+      <c r="J36" s="17"/>
     </row>
     <row r="37" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="24" t="s">
+      <c r="A37" s="23" t="s">
         <v>74</v>
       </c>
-      <c r="B37" s="18"/>
-      <c r="C37" s="18"/>
-      <c r="D37" s="18"/>
-      <c r="E37" s="18"/>
-      <c r="F37" s="17" t="s">
+      <c r="B37" s="17"/>
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="17"/>
+      <c r="F37" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="G37" s="18"/>
-      <c r="H37" s="18"/>
-      <c r="I37" s="18"/>
-      <c r="J37" s="18"/>
+      <c r="G37" s="17"/>
+      <c r="H37" s="17"/>
+      <c r="I37" s="17"/>
+      <c r="J37" s="17"/>
     </row>
     <row r="38" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="24" t="s">
+      <c r="A38" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="B38" s="18"/>
-      <c r="C38" s="18"/>
-      <c r="D38" s="18"/>
-      <c r="E38" s="18"/>
-      <c r="F38" s="14" t="s">
+      <c r="B38" s="17"/>
+      <c r="C38" s="17"/>
+      <c r="D38" s="17"/>
+      <c r="E38" s="17"/>
+      <c r="F38" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="G38" s="71" t="s">
+      <c r="G38" s="41" t="s">
         <v>90</v>
       </c>
-      <c r="H38" s="72"/>
-      <c r="I38" s="73" t="s">
+      <c r="H38" s="42"/>
+      <c r="I38" s="43" t="s">
         <v>91</v>
       </c>
-      <c r="J38" s="74"/>
+      <c r="J38" s="44"/>
     </row>
     <row r="39" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="14" t="s">
+      <c r="A39" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="B39" s="19" t="s">
+      <c r="B39" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="C39" s="19" t="s">
+      <c r="C39" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="D39" s="19" t="s">
+      <c r="D39" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="E39" s="19" t="s">
+      <c r="E39" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="F39" s="23" t="s">
+      <c r="F39" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="G39" s="27"/>
-      <c r="H39" s="28"/>
-      <c r="I39" s="27"/>
-      <c r="J39" s="28"/>
+      <c r="G39" s="26"/>
+      <c r="H39" s="27"/>
+      <c r="I39" s="26"/>
+      <c r="J39" s="27"/>
     </row>
     <row r="40" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="17" t="s">
+      <c r="A40" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="B40" s="18"/>
-      <c r="C40" s="18"/>
-      <c r="D40" s="18"/>
-      <c r="E40" s="18"/>
-      <c r="F40" s="17" t="s">
+      <c r="B40" s="17"/>
+      <c r="C40" s="17"/>
+      <c r="D40" s="17"/>
+      <c r="E40" s="17"/>
+      <c r="F40" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="G40" s="26"/>
-      <c r="H40" s="26"/>
-      <c r="I40" s="18"/>
-      <c r="J40" s="26"/>
+      <c r="G40" s="25"/>
+      <c r="H40" s="25"/>
+      <c r="I40" s="17"/>
+      <c r="J40" s="25"/>
     </row>
     <row r="41" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="17" t="s">
+      <c r="A41" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="B41" s="18"/>
-      <c r="C41" s="18"/>
-      <c r="D41" s="18"/>
-      <c r="E41" s="18"/>
-      <c r="F41" s="17" t="s">
+      <c r="B41" s="17"/>
+      <c r="C41" s="17"/>
+      <c r="D41" s="17"/>
+      <c r="E41" s="17"/>
+      <c r="F41" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="G41" s="33"/>
-      <c r="H41" s="34"/>
-      <c r="I41" s="33"/>
-      <c r="J41" s="34"/>
+      <c r="G41" s="45"/>
+      <c r="H41" s="46"/>
+      <c r="I41" s="45"/>
+      <c r="J41" s="46"/>
     </row>
     <row r="42" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="17" t="s">
+      <c r="A42" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="B42" s="18"/>
-      <c r="C42" s="18"/>
-      <c r="D42" s="18"/>
-      <c r="E42" s="18"/>
-      <c r="F42" s="17" t="s">
+      <c r="B42" s="17"/>
+      <c r="C42" s="17"/>
+      <c r="D42" s="17"/>
+      <c r="E42" s="17"/>
+      <c r="F42" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="G42" s="33"/>
-      <c r="H42" s="34"/>
-      <c r="I42" s="33"/>
-      <c r="J42" s="34"/>
+      <c r="G42" s="45"/>
+      <c r="H42" s="46"/>
+      <c r="I42" s="45"/>
+      <c r="J42" s="46"/>
     </row>
     <row r="43" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="17" t="s">
+      <c r="A43" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="B43" s="18"/>
-      <c r="C43" s="18"/>
-      <c r="D43" s="18"/>
-      <c r="E43" s="18"/>
-      <c r="F43" s="24" t="s">
+      <c r="B43" s="17"/>
+      <c r="C43" s="17"/>
+      <c r="D43" s="17"/>
+      <c r="E43" s="17"/>
+      <c r="F43" s="23" t="s">
         <v>60</v>
       </c>
-      <c r="G43" s="33"/>
-      <c r="H43" s="34"/>
-      <c r="I43" s="33"/>
-      <c r="J43" s="34"/>
+      <c r="G43" s="45"/>
+      <c r="H43" s="46"/>
+      <c r="I43" s="45"/>
+      <c r="J43" s="46"/>
     </row>
     <row r="44" spans="1:10" s="2" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="65" t="s">
+      <c r="A44" s="47" t="s">
         <v>61</v>
       </c>
-      <c r="B44" s="69"/>
-      <c r="C44" s="69"/>
-      <c r="D44" s="69"/>
-      <c r="E44" s="69"/>
-      <c r="F44" s="69"/>
-      <c r="G44" s="69"/>
-      <c r="H44" s="69"/>
-      <c r="I44" s="69"/>
-      <c r="J44" s="70"/>
+      <c r="B44" s="51"/>
+      <c r="C44" s="51"/>
+      <c r="D44" s="51"/>
+      <c r="E44" s="51"/>
+      <c r="F44" s="51"/>
+      <c r="G44" s="51"/>
+      <c r="H44" s="51"/>
+      <c r="I44" s="51"/>
+      <c r="J44" s="55"/>
     </row>
     <row r="45" spans="1:10" s="2" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="65" t="s">
+      <c r="A45" s="47" t="s">
         <v>62</v>
       </c>
-      <c r="B45" s="66"/>
-      <c r="C45" s="67"/>
-      <c r="D45" s="68" t="s">
+      <c r="B45" s="48"/>
+      <c r="C45" s="49"/>
+      <c r="D45" s="50" t="s">
         <v>59</v>
       </c>
-      <c r="E45" s="66"/>
-      <c r="F45" s="67"/>
-      <c r="G45" s="69" t="s">
+      <c r="E45" s="48"/>
+      <c r="F45" s="49"/>
+      <c r="G45" s="51" t="s">
         <v>63</v>
       </c>
-      <c r="H45" s="66"/>
-      <c r="I45" s="66"/>
-      <c r="J45" s="67"/>
+      <c r="H45" s="48"/>
+      <c r="I45" s="48"/>
+      <c r="J45" s="49"/>
     </row>
     <row r="46" spans="1:10" s="2" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="47" t="s">
+      <c r="A46" s="65" t="s">
         <v>77</v>
       </c>
-      <c r="B46" s="48"/>
-      <c r="C46" s="49"/>
-      <c r="D46" s="62" t="s">
+      <c r="B46" s="66"/>
+      <c r="C46" s="67"/>
+      <c r="D46" s="71" t="s">
         <v>64</v>
       </c>
-      <c r="E46" s="63"/>
-      <c r="F46" s="64"/>
-      <c r="G46" s="47" t="s">
+      <c r="E46" s="72"/>
+      <c r="F46" s="73"/>
+      <c r="G46" s="65" t="s">
         <v>105</v>
       </c>
-      <c r="H46" s="48"/>
-      <c r="I46" s="48"/>
-      <c r="J46" s="49"/>
+      <c r="H46" s="66"/>
+      <c r="I46" s="66"/>
+      <c r="J46" s="67"/>
     </row>
     <row r="47" spans="1:10" s="2" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="50" t="s">
+      <c r="A47" s="56" t="s">
         <v>78</v>
       </c>
-      <c r="B47" s="51"/>
-      <c r="C47" s="52"/>
-      <c r="D47" s="41" t="s">
+      <c r="B47" s="57"/>
+      <c r="C47" s="58"/>
+      <c r="D47" s="52" t="s">
         <v>65</v>
       </c>
-      <c r="E47" s="42"/>
-      <c r="F47" s="43"/>
-      <c r="G47" s="50" t="s">
+      <c r="E47" s="53"/>
+      <c r="F47" s="54"/>
+      <c r="G47" s="56" t="s">
         <v>106</v>
       </c>
-      <c r="H47" s="51"/>
-      <c r="I47" s="51"/>
-      <c r="J47" s="52"/>
+      <c r="H47" s="57"/>
+      <c r="I47" s="57"/>
+      <c r="J47" s="58"/>
     </row>
     <row r="48" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="50" t="s">
+      <c r="A48" s="56" t="s">
         <v>79</v>
       </c>
-      <c r="B48" s="51"/>
-      <c r="C48" s="52"/>
-      <c r="D48" s="41" t="s">
+      <c r="B48" s="57"/>
+      <c r="C48" s="58"/>
+      <c r="D48" s="52" t="s">
         <v>66</v>
       </c>
-      <c r="E48" s="42"/>
-      <c r="F48" s="43"/>
-      <c r="G48" s="50"/>
-      <c r="H48" s="51"/>
-      <c r="I48" s="51"/>
-      <c r="J48" s="52"/>
+      <c r="E48" s="53"/>
+      <c r="F48" s="54"/>
+      <c r="G48" s="56"/>
+      <c r="H48" s="57"/>
+      <c r="I48" s="57"/>
+      <c r="J48" s="58"/>
     </row>
     <row r="49" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="50" t="s">
+      <c r="A49" s="56" t="s">
         <v>82</v>
       </c>
-      <c r="B49" s="51"/>
-      <c r="C49" s="52"/>
-      <c r="D49" s="41" t="s">
+      <c r="B49" s="57"/>
+      <c r="C49" s="58"/>
+      <c r="D49" s="52" t="s">
         <v>67</v>
       </c>
-      <c r="E49" s="42"/>
-      <c r="F49" s="43"/>
-      <c r="G49" s="50"/>
-      <c r="H49" s="51"/>
-      <c r="I49" s="51"/>
-      <c r="J49" s="52"/>
+      <c r="E49" s="53"/>
+      <c r="F49" s="54"/>
+      <c r="G49" s="56"/>
+      <c r="H49" s="57"/>
+      <c r="I49" s="57"/>
+      <c r="J49" s="58"/>
     </row>
     <row r="50" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="50" t="s">
+      <c r="A50" s="56" t="s">
         <v>80</v>
       </c>
-      <c r="B50" s="51"/>
-      <c r="C50" s="52"/>
-      <c r="D50" s="41" t="s">
+      <c r="B50" s="57"/>
+      <c r="C50" s="58"/>
+      <c r="D50" s="52" t="s">
         <v>68</v>
       </c>
-      <c r="E50" s="42"/>
-      <c r="F50" s="43"/>
-      <c r="G50" s="53"/>
-      <c r="H50" s="54"/>
-      <c r="I50" s="54"/>
-      <c r="J50" s="55"/>
+      <c r="E50" s="53"/>
+      <c r="F50" s="54"/>
+      <c r="G50" s="59"/>
+      <c r="H50" s="60"/>
+      <c r="I50" s="60"/>
+      <c r="J50" s="61"/>
     </row>
     <row r="51" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="59" t="s">
+      <c r="A51" s="68" t="s">
         <v>81</v>
       </c>
-      <c r="B51" s="60"/>
-      <c r="C51" s="61"/>
-      <c r="D51" s="44" t="s">
+      <c r="B51" s="69"/>
+      <c r="C51" s="70"/>
+      <c r="D51" s="83" t="s">
         <v>69</v>
       </c>
-      <c r="E51" s="45"/>
-      <c r="F51" s="46"/>
-      <c r="G51" s="56" t="s">
+      <c r="E51" s="84"/>
+      <c r="F51" s="85"/>
+      <c r="G51" s="62" t="s">
         <v>83</v>
       </c>
-      <c r="H51" s="57"/>
-      <c r="I51" s="57"/>
-      <c r="J51" s="58"/>
+      <c r="H51" s="63"/>
+      <c r="I51" s="63"/>
+      <c r="J51" s="64"/>
     </row>
     <row r="52" spans="1:10" ht="18" x14ac:dyDescent="0.3">
-      <c r="A52" s="25" t="s">
+      <c r="A52" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="B52" s="35"/>
-      <c r="C52" s="36"/>
-      <c r="D52" s="36"/>
-      <c r="E52" s="36"/>
-      <c r="F52" s="36"/>
-      <c r="G52" s="36"/>
-      <c r="H52" s="36"/>
-      <c r="I52" s="36"/>
-      <c r="J52" s="37"/>
+      <c r="B52" s="77"/>
+      <c r="C52" s="78"/>
+      <c r="D52" s="78"/>
+      <c r="E52" s="78"/>
+      <c r="F52" s="78"/>
+      <c r="G52" s="78"/>
+      <c r="H52" s="78"/>
+      <c r="I52" s="78"/>
+      <c r="J52" s="79"/>
     </row>
     <row r="53" spans="1:10" ht="18" x14ac:dyDescent="0.3">
-      <c r="A53" s="38"/>
-      <c r="B53" s="39"/>
-      <c r="C53" s="39"/>
-      <c r="D53" s="39"/>
-      <c r="E53" s="39"/>
-      <c r="F53" s="39"/>
-      <c r="G53" s="39"/>
-      <c r="H53" s="39"/>
-      <c r="I53" s="39"/>
-      <c r="J53" s="40"/>
+      <c r="A53" s="80"/>
+      <c r="B53" s="81"/>
+      <c r="C53" s="81"/>
+      <c r="D53" s="81"/>
+      <c r="E53" s="81"/>
+      <c r="F53" s="81"/>
+      <c r="G53" s="81"/>
+      <c r="H53" s="81"/>
+      <c r="I53" s="81"/>
+      <c r="J53" s="82"/>
     </row>
     <row r="54" spans="1:10" ht="18" x14ac:dyDescent="0.3">
-      <c r="A54" s="38"/>
-      <c r="B54" s="39"/>
-      <c r="C54" s="39"/>
-      <c r="D54" s="39"/>
-      <c r="E54" s="39"/>
-      <c r="F54" s="39"/>
-      <c r="G54" s="39"/>
-      <c r="H54" s="39"/>
-      <c r="I54" s="39"/>
-      <c r="J54" s="40"/>
+      <c r="A54" s="80"/>
+      <c r="B54" s="81"/>
+      <c r="C54" s="81"/>
+      <c r="D54" s="81"/>
+      <c r="E54" s="81"/>
+      <c r="F54" s="81"/>
+      <c r="G54" s="81"/>
+      <c r="H54" s="81"/>
+      <c r="I54" s="81"/>
+      <c r="J54" s="82"/>
     </row>
     <row r="55" spans="1:10" ht="18" x14ac:dyDescent="0.3">
-      <c r="A55" s="30"/>
-      <c r="B55" s="31"/>
-      <c r="C55" s="31"/>
-      <c r="D55" s="31"/>
-      <c r="E55" s="31"/>
-      <c r="F55" s="31"/>
-      <c r="G55" s="31"/>
-      <c r="H55" s="31"/>
-      <c r="I55" s="31"/>
-      <c r="J55" s="32"/>
+      <c r="A55" s="74"/>
+      <c r="B55" s="75"/>
+      <c r="C55" s="75"/>
+      <c r="D55" s="75"/>
+      <c r="E55" s="75"/>
+      <c r="F55" s="75"/>
+      <c r="G55" s="75"/>
+      <c r="H55" s="75"/>
+      <c r="I55" s="75"/>
+      <c r="J55" s="76"/>
     </row>
   </sheetData>
-  <mergeCells count="64">
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="I7:J7"/>
+  <mergeCells count="65">
+    <mergeCell ref="A55:J55"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="B52:J52"/>
+    <mergeCell ref="A53:J53"/>
+    <mergeCell ref="A54:J54"/>
+    <mergeCell ref="D48:F48"/>
+    <mergeCell ref="D49:F49"/>
+    <mergeCell ref="D50:F50"/>
+    <mergeCell ref="D51:F51"/>
+    <mergeCell ref="G46:J46"/>
+    <mergeCell ref="G47:J47"/>
+    <mergeCell ref="G48:J48"/>
+    <mergeCell ref="G49:J49"/>
+    <mergeCell ref="G50:J50"/>
+    <mergeCell ref="G51:J51"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="A49:C49"/>
+    <mergeCell ref="A50:C50"/>
+    <mergeCell ref="A51:C51"/>
+    <mergeCell ref="D46:F46"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="D45:F45"/>
@@ -3189,38 +3202,23 @@
     <mergeCell ref="I42:J42"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="D11:E11"/>
-    <mergeCell ref="G48:J48"/>
-    <mergeCell ref="G49:J49"/>
-    <mergeCell ref="G50:J50"/>
-    <mergeCell ref="G51:J51"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="A46:C46"/>
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="A48:C48"/>
-    <mergeCell ref="A49:C49"/>
-    <mergeCell ref="A50:C50"/>
-    <mergeCell ref="A51:C51"/>
-    <mergeCell ref="D46:F46"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="A55:J55"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="B52:J52"/>
-    <mergeCell ref="A53:J53"/>
-    <mergeCell ref="A54:J54"/>
-    <mergeCell ref="D48:F48"/>
-    <mergeCell ref="D49:F49"/>
-    <mergeCell ref="D50:F50"/>
-    <mergeCell ref="D51:F51"/>
-    <mergeCell ref="G46:J46"/>
-    <mergeCell ref="G47:J47"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="I3:J3"/>
   </mergeCells>
   <dataValidations disablePrompts="1" count="1">
     <dataValidation showInputMessage="1" showErrorMessage="1" sqref="B6:F6" xr:uid="{00000000-0002-0000-0000-000000000000}"/>

</xml_diff>